<commit_message>
Remove spark imagery from music video plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H1B8siH6bLvLVTMznRPXcf
</commit_message>
<xml_diff>
--- a/mv-plan/原マシナリーMV企画.xlsx
+++ b/mv-plan/原マシナリーMV企画.xlsx
@@ -634,7 +634,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -663,7 +663,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>「削る、受け継ぐ、切り拓く」。金属を削る火花と工具の軌跡を共通のモチーフにして、1948年からの歴史・精度・素材・人・未来を一本の線でつなぐ。</t>
+          <t>「削る、受け継ぐ、切り拓く」。工具の軌跡（光の線）と削り出した面の金属光沢を共通のモチーフにして、1948年からの歴史・精度・素材・人・未来を一本の線でつなぐ。</t>
         </is>
       </c>
     </row>
@@ -675,7 +675,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>鉄の濃紺とスチールグレーを基調に、火花のアンバーを差し色にする。前半は重厚、サビで力強く、Cメロで温かく、ラストサビで最大の盛り上がりにする。</t>
+          <t>鉄の濃紺とスチールグレーを基調に、切削面の光沢を思わせるアンバーを差し色にする。前半は重厚、サビで力強く、Cメロで温かく、ラストサビで最大の盛り上がりにする。</t>
         </is>
       </c>
     </row>
@@ -779,25 +779,37 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="46" customHeight="1">
+    <row r="14" ht="20" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>重要な注意</t>
+          <t>表現の禁止事項</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>パートの開始・終了時刻は、曲の自動解析から出した推定値です。歌詞の文字起こしモデルがこの作業環境から使えなかったため、歌詞と時刻の対応は実際に聴いて確認・修正してください（「構成・絵コンテ」の青字を直すと、すべての時刻と長さが自動で再計算されます）。</t>
+          <t>火花の表現は使わない（CG・写真・効果音とも）。切削の表現は、工具の軌跡の線と金属の光沢で行う。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>重要な注意</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="inlineStr">
+        <is>
+          <t>パートの開始・終了時刻は、曲の自動解析から出した推定値です。歌詞の文字起こしモデルがこの作業環境から使えなかったため、歌詞と時刻の対応は実際に聴いて確認・修正してください（「構成・絵コンテ」の青字を直すと、すべての時刻と長さが自動で再計算されます）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="46" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>曲について</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>音源のメタデータに Suno（AI作曲サービス）で作成されたと記録されています。宣伝に使う場合は、作成時のプランの商用利用条件を確認してください。</t>
         </is>
@@ -960,19 +972,19 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>暗闇に鉄のブロック。エンドミルが入る瞬間に火花が散り、切削の軌跡が光の線になって「1948」を描く。</t>
+          <t>暗闇に鉄のブロック。エンドミルが静かに表面をなぞり、削られた面に金属の光沢が走る。工具の軌跡が光の線になって「1948」を描く。</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
           <t>・シェーダー（金属の質感）
-・パーティクル（火花）
+・光沢の走り（シェーダー）
 ・線を描く（SVG）</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>拍ごとに火花の量が増える。最後の拍で「1948」が完成</t>
+          <t>拍ごとに軌跡の線が1本ずつ増える。最後の拍で「1948」が完成</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
@@ -1215,13 +1227,13 @@
           <t>・1文字ずつ出現
 ・拍ごとのカット
 ・3D モデル
-・パーティクル（火花）
+・光沢の走り（シェーダー）
 ・線を描く（SVG）</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>4つの力＝4拍。「原マシナリー」でロゴ確定＋火花</t>
+          <t>4つの力＝4拍。「原マシナリー」でロゴ確定＋光沢がロゴを横切る</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
@@ -1462,7 +1474,7 @@
 ・拍ごとのカット
 ・3D モデル
 ・Lottie アイコン
-・パーティクル（火花）</t>
+・光沢の走り（シェーダー）</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
@@ -1578,7 +1590,7 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>最大の盛り上がり。年号カウンターが 1948 → 2048（100年企業）。全写真を拍ごとに高速モンタージュ。3D ロゴが回転し、「切り拓け」で画面全体が切削されて光が差し込む。紙吹雪と火花。</t>
+          <t>最大の盛り上がり。年号カウンターが 1948 → 2048（100年企業）。全写真を拍ごとに高速モンタージュ。3D ロゴが回転し、「切り拓け」で画面全体が切削されて光が差し込む。紙吹雪と、ロゴを走る金属の光沢。</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
@@ -1587,7 +1599,7 @@
 ・拍ごとのカット
 ・3D モデル
 ・シェーダー（金属の質感）
-・パーティクル（火花）
+・光沢の走り（シェーダー）
 ・紙吹雪
 ・1文字ずつ出現</t>
         </is>
@@ -1643,14 +1655,14 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>静かに火花が消え、ロゴとスローガン「受け継ぐ技術 挑み続ける心」。最後にURLを表示してフェードアウト。</t>
+          <t>工具の軌跡の線が静かに消え、ロゴとスローガン「受け継ぐ技術 挑み続ける心」。最後にURLを表示してフェードアウト。</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
           <t>・線を描く（SVG）
 ・フェード
-・パーティクル（火花）</t>
+・光沢の走り（シェーダー）</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
@@ -4562,7 +4574,7 @@
     <row r="6">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>パーティクル（火花）</t>
+          <t>光沢の走り（シェーダー）</t>
         </is>
       </c>
       <c r="B6" s="12" t="inlineStr">
@@ -5607,7 +5619,7 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>火花・切削の瞬間があると最適</t>
+          <t>切削の瞬間や仕上げ面のアップがあると最適</t>
         </is>
       </c>
       <c r="E9" s="28" t="inlineStr">

</xml_diff>